<commit_message>
Harden task: strip costing memo to principles, add re-created/rebuilt id traps, retune labour so the decision is contestable
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015zvfotZNd3VuWwxgMsj6vJ
</commit_message>
<xml_diff>
--- a/project_mark_task/inputs/client_master.xlsx
+++ b/project_mark_task/inputs/client_master.xlsx
@@ -461,7 +461,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -489,7 +489,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>active</t>
+          <t xml:space="preserve">Active </t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -545,7 +545,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>CHURNED</t>
+          <t>Inactive</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -605,7 +605,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Active </t>
+          <t>Active</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -633,7 +633,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Active </t>
+          <t>Active</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -644,7 +644,7 @@
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Northgate Automations Ltd</t>
+          <t>Northgate Labs GmbH</t>
         </is>
       </c>
     </row>
@@ -672,7 +672,7 @@
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Northgate Automations Ltd</t>
+          <t>Northgate Labs GmbH</t>
         </is>
       </c>
     </row>
@@ -689,7 +689,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t xml:space="preserve">Active </t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -717,7 +717,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>CHURNED</t>
+          <t>churned</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -749,7 +749,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>active</t>
+          <t xml:space="preserve">Active </t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -777,7 +777,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -805,7 +805,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>active</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -816,7 +816,7 @@
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Northgate Automations Ltd</t>
+          <t>Northgate Labs GmbH</t>
         </is>
       </c>
     </row>
@@ -833,7 +833,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -861,7 +861,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Churned</t>
+          <t>Inactive</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -871,12 +871,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Jun 06, 2025</t>
+          <t>2025-06-06</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Northgate Labs GmbH</t>
+          <t>Northgate Automations Ltd</t>
         </is>
       </c>
     </row>
@@ -921,7 +921,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t xml:space="preserve">Active </t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -977,7 +977,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1005,7 +1005,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>active</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1016,7 +1016,7 @@
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Northgate Automations Ltd</t>
+          <t>Northgate Labs GmbH</t>
         </is>
       </c>
     </row>
@@ -1033,7 +1033,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1061,7 +1061,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>churned</t>
+          <t>Churned</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1093,7 +1093,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t xml:space="preserve">Active </t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1149,7 +1149,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>active</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1177,7 +1177,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Active </t>
+          <t>active</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1205,7 +1205,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Active </t>
+          <t>Active</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1216,7 +1216,7 @@
       <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Northgate Automations Ltd</t>
+          <t>Northgate Labs GmbH</t>
         </is>
       </c>
     </row>
@@ -1233,7 +1233,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Active </t>
+          <t>active</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">

</xml_diff>

<commit_message>
v3: add helper sub-flow workflows (catalog notes only), retune pricing/hours, update reference outputs and rubric
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015zvfotZNd3VuWwxgMsj6vJ
</commit_message>
<xml_diff>
--- a/project_mark_task/inputs/client_master.xlsx
+++ b/project_mark_task/inputs/client_master.xlsx
@@ -500,7 +500,7 @@
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Northgate Labs GmbH</t>
+          <t>Northgate Automations Ltd</t>
         </is>
       </c>
     </row>
@@ -545,7 +545,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Inactive</t>
+          <t>CHURNED</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -555,7 +555,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Jul 10, 2025</t>
+          <t>10/07/2025</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -588,7 +588,7 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Northgate Labs GmbH</t>
+          <t>Northgate Automations Ltd</t>
         </is>
       </c>
     </row>
@@ -605,7 +605,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>active</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -616,7 +616,7 @@
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Northgate Labs GmbH</t>
+          <t>Northgate Automations Ltd</t>
         </is>
       </c>
     </row>
@@ -644,7 +644,7 @@
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Northgate Labs GmbH</t>
+          <t>Northgate Automations Ltd</t>
         </is>
       </c>
     </row>
@@ -661,7 +661,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t xml:space="preserve">Active </t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -689,7 +689,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Active </t>
+          <t>Active</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -717,7 +717,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>churned</t>
+          <t>CHURNED</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -727,7 +727,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>18/03/2025</t>
+          <t>Mar 18, 2025</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -777,7 +777,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t xml:space="preserve">Active </t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -816,7 +816,7 @@
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Northgate Labs GmbH</t>
+          <t>Northgate Automations Ltd</t>
         </is>
       </c>
     </row>
@@ -833,7 +833,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t xml:space="preserve">Active </t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -871,7 +871,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2025-06-06</t>
+          <t>Jun 06, 2025</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -904,7 +904,7 @@
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Northgate Labs GmbH</t>
+          <t>Northgate Automations Ltd</t>
         </is>
       </c>
     </row>
@@ -921,7 +921,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Active </t>
+          <t>Active</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -949,7 +949,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>active</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -960,7 +960,7 @@
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Northgate Automations Ltd</t>
+          <t>Northgate Labs GmbH</t>
         </is>
       </c>
     </row>
@@ -1005,7 +1005,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>active</t>
+          <t xml:space="preserve">Active </t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1033,7 +1033,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>active</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1061,7 +1061,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Churned</t>
+          <t>churned</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1076,7 +1076,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Northgate Labs GmbH</t>
+          <t>Northgate Automations Ltd</t>
         </is>
       </c>
     </row>
@@ -1093,7 +1093,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Active </t>
+          <t>Active</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1132,7 +1132,7 @@
       <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Northgate Labs GmbH</t>
+          <t>Northgate Automations Ltd</t>
         </is>
       </c>
     </row>
@@ -1149,7 +1149,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>active</t>
+          <t xml:space="preserve">Active </t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1160,7 +1160,7 @@
       <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Northgate Automations Ltd</t>
+          <t>Northgate Labs GmbH</t>
         </is>
       </c>
     </row>
@@ -1205,7 +1205,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t xml:space="preserve">Active </t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1233,7 +1233,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>active</t>
+          <t xml:space="preserve">Active </t>
         </is>
       </c>
       <c r="D29" t="inlineStr">

</xml_diff>

<commit_message>
WIP v4: Zapier plan-upgrade clause and one-off backfill bursts
Rubric, reference PDF and checkpoints still reflect v3 and need regenerating after retuning.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015zvfotZNd3VuWwxgMsj6vJ
</commit_message>
<xml_diff>
--- a/project_mark_task/inputs/client_master.xlsx
+++ b/project_mark_task/inputs/client_master.xlsx
@@ -461,7 +461,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>active</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -489,7 +489,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Active </t>
+          <t>active</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -500,7 +500,7 @@
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Northgate Automations Ltd</t>
+          <t>Northgate Labs GmbH</t>
         </is>
       </c>
     </row>
@@ -555,7 +555,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>10/07/2025</t>
+          <t>Jul 10, 2025</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -577,7 +577,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>active</t>
+          <t xml:space="preserve">Active </t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -588,7 +588,7 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Northgate Automations Ltd</t>
+          <t>Northgate Labs GmbH</t>
         </is>
       </c>
     </row>
@@ -605,7 +605,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -633,7 +633,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t xml:space="preserve">Active </t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -661,7 +661,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Active </t>
+          <t>Active</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -689,7 +689,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t xml:space="preserve">Active </t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -777,7 +777,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Active </t>
+          <t>Active</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -805,7 +805,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -816,7 +816,7 @@
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Northgate Automations Ltd</t>
+          <t>Northgate Labs GmbH</t>
         </is>
       </c>
     </row>
@@ -833,7 +833,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Active </t>
+          <t>active</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -844,7 +844,7 @@
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Northgate Labs GmbH</t>
+          <t>Northgate Automations Ltd</t>
         </is>
       </c>
     </row>
@@ -871,7 +871,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Jun 06, 2025</t>
+          <t>2025-06-06</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -893,7 +893,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>active</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -904,7 +904,7 @@
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Northgate Automations Ltd</t>
+          <t>Northgate Labs GmbH</t>
         </is>
       </c>
     </row>
@@ -949,7 +949,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -960,7 +960,7 @@
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Northgate Labs GmbH</t>
+          <t>Northgate Automations Ltd</t>
         </is>
       </c>
     </row>
@@ -1005,7 +1005,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Active </t>
+          <t>active</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1016,7 +1016,7 @@
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Northgate Labs GmbH</t>
+          <t>Northgate Automations Ltd</t>
         </is>
       </c>
     </row>
@@ -1033,7 +1033,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>active</t>
+          <t xml:space="preserve">Active </t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1044,7 +1044,7 @@
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Northgate Automations Ltd</t>
+          <t>Northgate Labs GmbH</t>
         </is>
       </c>
     </row>
@@ -1061,7 +1061,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>churned</t>
+          <t>CHURNED</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1071,7 +1071,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>12/07/2025</t>
+          <t>2025-07-12</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1093,7 +1093,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>active</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1104,7 +1104,7 @@
       <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Northgate Automations Ltd</t>
+          <t>Northgate Labs GmbH</t>
         </is>
       </c>
     </row>
@@ -1149,7 +1149,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Active </t>
+          <t>Active</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1177,7 +1177,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1205,7 +1205,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Active </t>
+          <t>active</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1233,7 +1233,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Active </t>
+          <t>Active</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1244,7 +1244,7 @@
       <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Northgate Automations Ltd</t>
+          <t>Northgate Labs GmbH</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
v5: Zapier export column drift, re-signed clients, more incidents, Make negotiated rate; retuned costs, rubric v5, scorer
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015zvfotZNd3VuWwxgMsj6vJ
</commit_message>
<xml_diff>
--- a/project_mark_task/inputs/client_master.xlsx
+++ b/project_mark_task/inputs/client_master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -461,7 +461,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -489,7 +489,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>active</t>
+          <t xml:space="preserve">Active </t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -500,7 +500,7 @@
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Northgate Labs GmbH</t>
+          <t>Northgate Automations Ltd</t>
         </is>
       </c>
     </row>
@@ -545,7 +545,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>CHURNED</t>
+          <t>churned</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -555,7 +555,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Jul 10, 2025</t>
+          <t>2025-07-10</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -577,7 +577,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Active </t>
+          <t>Active</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -588,7 +588,7 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Northgate Labs GmbH</t>
+          <t>Northgate Automations Ltd</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Active </t>
+          <t>Active</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -717,7 +717,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>CHURNED</t>
+          <t>Inactive</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -727,7 +727,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Mar 18, 2025</t>
+          <t>18/03/2025</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -749,7 +749,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Active </t>
+          <t>Active</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -777,7 +777,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>active</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -788,7 +788,7 @@
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Northgate Automations Ltd</t>
+          <t>Northgate Labs GmbH</t>
         </is>
       </c>
     </row>
@@ -816,7 +816,7 @@
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Northgate Labs GmbH</t>
+          <t>Northgate Automations Ltd</t>
         </is>
       </c>
     </row>
@@ -833,7 +833,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>active</t>
+          <t xml:space="preserve">Active </t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -844,7 +844,7 @@
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Northgate Automations Ltd</t>
+          <t>Northgate Labs GmbH</t>
         </is>
       </c>
     </row>
@@ -861,7 +861,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Inactive</t>
+          <t>CHURNED</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -871,7 +871,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2025-06-06</t>
+          <t>Jun 06, 2025</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -921,7 +921,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t xml:space="preserve">Active </t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1005,7 +1005,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>active</t>
+          <t xml:space="preserve">Active </t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1033,7 +1033,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Active </t>
+          <t>active</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1044,7 +1044,7 @@
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Northgate Labs GmbH</t>
+          <t>Northgate Automations Ltd</t>
         </is>
       </c>
     </row>
@@ -1061,7 +1061,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>CHURNED</t>
+          <t>Inactive</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1071,7 +1071,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2025-07-12</t>
+          <t>Jul 12, 2025</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1093,7 +1093,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>active</t>
+          <t xml:space="preserve">Active </t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1104,7 +1104,7 @@
       <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Northgate Labs GmbH</t>
+          <t>Northgate Automations Ltd</t>
         </is>
       </c>
     </row>
@@ -1121,7 +1121,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t xml:space="preserve">Active </t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1132,7 +1132,7 @@
       <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Northgate Automations Ltd</t>
+          <t>Northgate Labs GmbH</t>
         </is>
       </c>
     </row>
@@ -1160,7 +1160,7 @@
       <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Northgate Labs GmbH</t>
+          <t>Northgate Automations Ltd</t>
         </is>
       </c>
     </row>
@@ -1177,7 +1177,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t xml:space="preserve">Active </t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1188,7 +1188,7 @@
       <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Northgate Automations Ltd</t>
+          <t>Northgate Labs GmbH</t>
         </is>
       </c>
     </row>
@@ -1205,7 +1205,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>active</t>
+          <t xml:space="preserve">Active </t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1216,7 +1216,7 @@
       <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Northgate Labs GmbH</t>
+          <t>Northgate Automations Ltd</t>
         </is>
       </c>
     </row>
@@ -1245,6 +1245,62 @@
       <c r="F29" t="inlineStr">
         <is>
           <t>Northgate Labs GmbH</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>CL-029</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Nimbus Cloud Print (2025 contract)</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>2025-07-11</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Northgate Automations Ltd</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>CL-030</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Tidewater Marine Supply (2025 contract)</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>2025-03-19</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Northgate Automations Ltd</t>
         </is>
       </c>
     </row>

</xml_diff>